<commit_message>
Rebuild 2026-06-08 report with full Luminor fund set
</commit_message>
<xml_diff>
--- a/docs/pension_data_combined_2026-06-08.xlsx
+++ b/docs/pension_data_combined_2026-06-08.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D52"/>
+  <dimension ref="A1:D55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40.12" customWidth="1" min="1" max="1"/>
@@ -466,14 +466,14 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1.15</v>
+        <v>1.1704</v>
       </c>
       <c r="D3" t="n">
-        <v>2042075.34</v>
+        <v>2078237.42</v>
       </c>
     </row>
     <row r="4">
@@ -484,14 +484,14 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1.1774</v>
+        <v>1.1815</v>
       </c>
       <c r="D4" t="n">
-        <v>35053518.08</v>
+        <v>35023908.84</v>
       </c>
     </row>
     <row r="5">
@@ -502,14 +502,14 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1.4392</v>
+        <v>1.45</v>
       </c>
       <c r="D5" t="n">
-        <v>185050070.62</v>
+        <v>186924046.34</v>
       </c>
     </row>
     <row r="6">
@@ -520,14 +520,14 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1.938</v>
+        <v>1.965</v>
       </c>
       <c r="D6" t="n">
-        <v>213255700.33</v>
+        <v>216247291.5</v>
       </c>
     </row>
     <row r="7">
@@ -538,14 +538,14 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2.1969</v>
+        <v>2.2323</v>
       </c>
       <c r="D7" t="n">
-        <v>218096205.65</v>
+        <v>221610375.34</v>
       </c>
     </row>
     <row r="8">
@@ -556,14 +556,14 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>2.2328</v>
+        <v>2.2687</v>
       </c>
       <c r="D8" t="n">
-        <v>176784811.56</v>
+        <v>179576437.99</v>
       </c>
     </row>
     <row r="9">
@@ -574,14 +574,14 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>2.2245</v>
+        <v>2.2645</v>
       </c>
       <c r="D9" t="n">
-        <v>96338968.45</v>
+        <v>98076736.56999999</v>
       </c>
     </row>
     <row r="10">
@@ -592,14 +592,14 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>2.2102</v>
+        <v>2.2478</v>
       </c>
       <c r="D10" t="n">
-        <v>37357029.04</v>
+        <v>37988553.27</v>
       </c>
     </row>
     <row r="11">
@@ -617,14 +617,14 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1.2026</v>
+        <v>1.2182</v>
       </c>
       <c r="D12" t="n">
-        <v>2994691.23</v>
+        <v>3035491.03</v>
       </c>
     </row>
     <row r="13">
@@ -635,14 +635,14 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>2.2893</v>
+        <v>2.3105</v>
       </c>
       <c r="D13" t="n">
-        <v>35707593.64</v>
+        <v>36044763.78</v>
       </c>
     </row>
     <row r="14">
@@ -653,14 +653,14 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>2.2749</v>
+        <v>2.2945</v>
       </c>
       <c r="D14" t="n">
-        <v>125173158.84</v>
+        <v>126263532.52</v>
       </c>
     </row>
     <row r="15">
@@ -671,14 +671,14 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>2.2794</v>
+        <v>2.3</v>
       </c>
       <c r="D15" t="n">
-        <v>231455055.7</v>
+        <v>233548440.99</v>
       </c>
     </row>
     <row r="16">
@@ -689,14 +689,14 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>2.2596</v>
+        <v>2.2782</v>
       </c>
       <c r="D16" t="n">
-        <v>226266873.56</v>
+        <v>228191611.64</v>
       </c>
     </row>
     <row r="17">
@@ -707,14 +707,14 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1.9604</v>
+        <v>1.9705</v>
       </c>
       <c r="D17" t="n">
-        <v>168375231.41</v>
+        <v>169286229.96</v>
       </c>
     </row>
     <row r="18">
@@ -725,14 +725,14 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>1.5478</v>
+        <v>1.5535</v>
       </c>
       <c r="D18" t="n">
-        <v>111146215.79</v>
+        <v>111769386.93</v>
       </c>
     </row>
     <row r="19">
@@ -743,14 +743,14 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>1.249</v>
+        <v>1.2516</v>
       </c>
       <c r="D19" t="n">
-        <v>17332150.96</v>
+        <v>17432469.21</v>
       </c>
     </row>
     <row r="20">
@@ -768,14 +768,14 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>1.185</v>
+        <v>1.2019</v>
       </c>
       <c r="D21" t="n">
-        <v>4263676.6763</v>
+        <v>4352757.0641</v>
       </c>
     </row>
     <row r="22">
@@ -786,14 +786,14 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>1.559</v>
+        <v>1.5813</v>
       </c>
       <c r="D22" t="n">
-        <v>27289633.4609</v>
+        <v>27661793.6232</v>
       </c>
     </row>
     <row r="23">
@@ -804,14 +804,14 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1.5552</v>
+        <v>1.5775</v>
       </c>
       <c r="D23" t="n">
-        <v>49288764.4671</v>
+        <v>49955360.9916</v>
       </c>
     </row>
     <row r="24">
@@ -822,14 +822,14 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>1.5641</v>
+        <v>1.5865</v>
       </c>
       <c r="D24" t="n">
-        <v>60980023.7131</v>
+        <v>61824051.0241</v>
       </c>
     </row>
     <row r="25">
@@ -840,14 +840,14 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1.5568</v>
+        <v>1.579</v>
       </c>
       <c r="D25" t="n">
-        <v>55722707.5956</v>
+        <v>56440730.1901</v>
       </c>
     </row>
     <row r="26">
@@ -858,14 +858,14 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>1.542</v>
+        <v>1.5621</v>
       </c>
       <c r="D26" t="n">
-        <v>36780653.5596</v>
+        <v>37330300.5932</v>
       </c>
     </row>
     <row r="27">
@@ -876,14 +876,14 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1.2619</v>
+        <v>1.2663</v>
       </c>
       <c r="D27" t="n">
-        <v>10725254.722</v>
+        <v>10806070.7884</v>
       </c>
     </row>
     <row r="28">
@@ -894,14 +894,14 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1.091</v>
+        <v>1.0921</v>
       </c>
       <c r="D28" t="n">
-        <v>1761156.5143</v>
+        <v>1736747.3953</v>
       </c>
     </row>
     <row r="29">
@@ -914,7 +914,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Luminor 1982-1988 tikslinės grupės pensijų fondas</t>
+          <t>Luminor 2003-2009 tikslinės grupės pensijų fondas</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -923,16 +923,16 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>2.2345</v>
+        <v>1.1688</v>
       </c>
       <c r="D30" t="n">
-        <v>116064081.95</v>
+        <v>3715262</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Luminor 1975-1981 tikslinės grupės pensijų fondas</t>
+          <t>Luminor 1996-2002 tikslinės grupės pensijų fondas</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -941,16 +941,16 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>2.2327</v>
+        <v>2.2639</v>
       </c>
       <c r="D31" t="n">
-        <v>125691384.1</v>
+        <v>21778247</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Luminor 1968-1974 tikslinės grupės pensijų fondas</t>
+          <t>Luminor 1989-1995 tikslinės grupės pensijų fondas</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -959,16 +959,16 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>2.0397</v>
+        <v>2.2507</v>
       </c>
       <c r="D32" t="n">
-        <v>110911258.69</v>
+        <v>60362344</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Luminor 1961-1967 tikslinės grupės pensijų fondas</t>
+          <t>Luminor 1982-1988 tikslinės grupės pensijų fondas</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -977,16 +977,16 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>1.5701</v>
+        <v>2.2345</v>
       </c>
       <c r="D33" t="n">
-        <v>88882605.02</v>
+        <v>116064082</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Luminor pensijų turto išsaugojimo fondas</t>
+          <t>Luminor 1975-1981 tikslinės grupės pensijų fondas</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -995,23 +995,34 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>1.1651</v>
+        <v>2.2327</v>
       </c>
       <c r="D34" t="n">
-        <v>14549017.81</v>
+        <v>125691384</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>SEB</t>
-        </is>
+          <t>Luminor 1968-1974 tikslinės grupės pensijų fondas</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>2.0397</v>
+      </c>
+      <c r="D35" t="n">
+        <v>110911259</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>SEB pensija 2003-2009</t>
+          <t>Luminor 1961-1967 tikslinės grupės pensijų fondas</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1020,16 +1031,16 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>1.1619</v>
+        <v>1.5701</v>
       </c>
       <c r="D36" t="n">
-        <v>2526191</v>
+        <v>88882605</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>SEB pensija 1996-2002</t>
+          <t>Luminor pensijų turto išsaugojimo fondas</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1038,269 +1049,312 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>2.3128</v>
+        <v>1.1651</v>
       </c>
       <c r="D37" t="n">
-        <v>46481585</v>
+        <v>14549018</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>SEB pensija 1989-1995</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>2026-06-08</t>
-        </is>
-      </c>
-      <c r="C38" t="n">
-        <v>2.292</v>
-      </c>
-      <c r="D38" t="n">
-        <v>153000174</v>
+          <t>SEB</t>
+        </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>SEB pensija 1982-1988</t>
+          <t>SEB pensija 2003-2009</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>2.2962</v>
+        <v>1.1801</v>
       </c>
       <c r="D39" t="n">
-        <v>371573320</v>
+        <v>2565873</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>SEB pensija 1975-1981</t>
+          <t>SEB pensija 1996-2002</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>2.3289</v>
+        <v>2.3476</v>
       </c>
       <c r="D40" t="n">
-        <v>473974390</v>
+        <v>47200339</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>SEB pensija 1968-1974</t>
+          <t>SEB pensija 1989-1995</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>2.0196</v>
+        <v>2.3266</v>
       </c>
       <c r="D41" t="n">
-        <v>389760718</v>
+        <v>155242467</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>SEB pensija 1961-1967</t>
+          <t>SEB pensija 1982-1988</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>1.5462</v>
+        <v>2.3307</v>
       </c>
       <c r="D42" t="n">
-        <v>292027629</v>
+        <v>377114950</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>SEB turto išsaugojimo fondas</t>
+          <t>SEB pensija 1975-1981</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>1.2087</v>
+        <v>2.3626</v>
       </c>
       <c r="D43" t="n">
-        <v>58083644</v>
+        <v>480857177</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>SWEDBANK</t>
-        </is>
+          <t>SEB pensija 1968-1974</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>2.0391</v>
+      </c>
+      <c r="D44" t="n">
+        <v>393620386</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Pensija 2003-2009</t>
+          <t>SEB pensija 1961-1967</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>1.1194</v>
+        <v>1.5548</v>
       </c>
       <c r="D45" t="n">
-        <v>3684949.21</v>
+        <v>294503324</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Pensija 1996-2002</t>
+          <t>SEB turto išsaugojimo fondas</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>2.1083</v>
+        <v>1.2134</v>
       </c>
       <c r="D46" t="n">
-        <v>82675842.75</v>
+        <v>58226459</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Pensija 1989-1995</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>2026-06-08</t>
-        </is>
-      </c>
-      <c r="C47" t="n">
-        <v>2.1266</v>
-      </c>
-      <c r="D47" t="n">
-        <v>265722392.32</v>
+          <t>SWEDBANK</t>
+        </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Pensija 1982-1988</t>
+          <t>Pensija 2003-2009</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>2.1441</v>
+        <v>1.1389</v>
       </c>
       <c r="D48" t="n">
-        <v>405199363.07</v>
+        <v>3755721.97</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Pensija 1975-1981</t>
+          <t>Pensija 1996-2002</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>2.1494</v>
+        <v>2.1417</v>
       </c>
       <c r="D49" t="n">
-        <v>493905901.26</v>
+        <v>83948772.52</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Pensija 1968-1974</t>
+          <t>Pensija 1989-1995</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>1.9491</v>
+        <v>2.1606</v>
       </c>
       <c r="D50" t="n">
-        <v>463508263.09</v>
+        <v>269986593.2</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Pensija 1961-1967</t>
+          <t>Pensija 1982-1988</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>1.5353</v>
+        <v>2.1784</v>
       </c>
       <c r="D51" t="n">
-        <v>366178131.11</v>
+        <v>411711586.5</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
+          <t>Pensija 1975-1981</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>2.1816</v>
+      </c>
+      <c r="D52" t="n">
+        <v>501328438.3</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Pensija 1968-1974</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>1.9678</v>
+      </c>
+      <c r="D53" t="n">
+        <v>468010624.1</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Pensija 1961-1967</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>1.5442</v>
+      </c>
+      <c r="D54" t="n">
+        <v>368167097.8</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
           <t>Turto išsaugojimo pensijų fondas</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>2026-06-08</t>
-        </is>
-      </c>
-      <c r="C52" t="n">
-        <v>1.1983</v>
-      </c>
-      <c r="D52" t="n">
-        <v>67984412.33</v>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>1.2046</v>
+      </c>
+      <c r="D55" t="n">
+        <v>68503948.73999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix 06-08 report dates across all providers
</commit_message>
<xml_diff>
--- a/docs/pension_data_combined_2026-06-08.xlsx
+++ b/docs/pension_data_combined_2026-06-08.xlsx
@@ -466,14 +466,14 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>1.1704</v>
+        <v>1.15</v>
       </c>
       <c r="D3" t="n">
-        <v>2078237.42</v>
+        <v>2042075.34</v>
       </c>
     </row>
     <row r="4">
@@ -484,14 +484,14 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1.1815</v>
+        <v>1.1774</v>
       </c>
       <c r="D4" t="n">
-        <v>35023908.84</v>
+        <v>35053518.08</v>
       </c>
     </row>
     <row r="5">
@@ -502,14 +502,14 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1.45</v>
+        <v>1.4392</v>
       </c>
       <c r="D5" t="n">
-        <v>186924046.34</v>
+        <v>185050070.62</v>
       </c>
     </row>
     <row r="6">
@@ -520,14 +520,14 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>1.965</v>
+        <v>1.938</v>
       </c>
       <c r="D6" t="n">
-        <v>216247291.5</v>
+        <v>213255700.33</v>
       </c>
     </row>
     <row r="7">
@@ -538,14 +538,14 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2.2323</v>
+        <v>2.1969</v>
       </c>
       <c r="D7" t="n">
-        <v>221610375.34</v>
+        <v>218096205.65</v>
       </c>
     </row>
     <row r="8">
@@ -556,14 +556,14 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>2.2687</v>
+        <v>2.2328</v>
       </c>
       <c r="D8" t="n">
-        <v>179576437.99</v>
+        <v>176784811.56</v>
       </c>
     </row>
     <row r="9">
@@ -574,14 +574,14 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>2.2645</v>
+        <v>2.2245</v>
       </c>
       <c r="D9" t="n">
-        <v>98076736.56999999</v>
+        <v>96338968.45</v>
       </c>
     </row>
     <row r="10">
@@ -592,14 +592,14 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>2.2478</v>
+        <v>2.2102</v>
       </c>
       <c r="D10" t="n">
-        <v>37988553.27</v>
+        <v>37357029.04</v>
       </c>
     </row>
     <row r="11">
@@ -617,14 +617,14 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1.2182</v>
+        <v>1.2026</v>
       </c>
       <c r="D12" t="n">
-        <v>3035491.03</v>
+        <v>2994691.23</v>
       </c>
     </row>
     <row r="13">
@@ -635,14 +635,14 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>2.3105</v>
+        <v>2.2893</v>
       </c>
       <c r="D13" t="n">
-        <v>36044763.78</v>
+        <v>35707593.64</v>
       </c>
     </row>
     <row r="14">
@@ -653,14 +653,14 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>2.2945</v>
+        <v>2.2749</v>
       </c>
       <c r="D14" t="n">
-        <v>126263532.52</v>
+        <v>125173158.84</v>
       </c>
     </row>
     <row r="15">
@@ -671,14 +671,14 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>2.3</v>
+        <v>2.2794</v>
       </c>
       <c r="D15" t="n">
-        <v>233548440.99</v>
+        <v>231455055.7</v>
       </c>
     </row>
     <row r="16">
@@ -689,14 +689,14 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>2.2782</v>
+        <v>2.2596</v>
       </c>
       <c r="D16" t="n">
-        <v>228191611.64</v>
+        <v>226266873.56</v>
       </c>
     </row>
     <row r="17">
@@ -707,14 +707,14 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1.9705</v>
+        <v>1.9604</v>
       </c>
       <c r="D17" t="n">
-        <v>169286229.96</v>
+        <v>168375231.41</v>
       </c>
     </row>
     <row r="18">
@@ -725,14 +725,14 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>1.5535</v>
+        <v>1.5478</v>
       </c>
       <c r="D18" t="n">
-        <v>111769386.93</v>
+        <v>111146215.79</v>
       </c>
     </row>
     <row r="19">
@@ -743,14 +743,14 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>1.2516</v>
+        <v>1.249</v>
       </c>
       <c r="D19" t="n">
-        <v>17432469.21</v>
+        <v>17332150.96</v>
       </c>
     </row>
     <row r="20">
@@ -768,14 +768,14 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>1.2019</v>
+        <v>1.185</v>
       </c>
       <c r="D21" t="n">
-        <v>4352757.0641</v>
+        <v>4263676.6763</v>
       </c>
     </row>
     <row r="22">
@@ -786,14 +786,14 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>1.5813</v>
+        <v>1.559</v>
       </c>
       <c r="D22" t="n">
-        <v>27661793.6232</v>
+        <v>27289633.4609</v>
       </c>
     </row>
     <row r="23">
@@ -804,14 +804,14 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1.5775</v>
+        <v>1.5552</v>
       </c>
       <c r="D23" t="n">
-        <v>49955360.9916</v>
+        <v>49288764.4671</v>
       </c>
     </row>
     <row r="24">
@@ -822,14 +822,14 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>1.5865</v>
+        <v>1.5641</v>
       </c>
       <c r="D24" t="n">
-        <v>61824051.0241</v>
+        <v>60980023.7131</v>
       </c>
     </row>
     <row r="25">
@@ -840,14 +840,14 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1.579</v>
+        <v>1.5568</v>
       </c>
       <c r="D25" t="n">
-        <v>56440730.1901</v>
+        <v>55722707.5956</v>
       </c>
     </row>
     <row r="26">
@@ -858,14 +858,14 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>1.5621</v>
+        <v>1.542</v>
       </c>
       <c r="D26" t="n">
-        <v>37330300.5932</v>
+        <v>36780653.5596</v>
       </c>
     </row>
     <row r="27">
@@ -876,14 +876,14 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1.2663</v>
+        <v>1.2619</v>
       </c>
       <c r="D27" t="n">
-        <v>10806070.7884</v>
+        <v>10725254.722</v>
       </c>
     </row>
     <row r="28">
@@ -894,14 +894,14 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1.0921</v>
+        <v>1.091</v>
       </c>
       <c r="D28" t="n">
-        <v>1736747.3953</v>
+        <v>1761156.5143</v>
       </c>
     </row>
     <row r="29">
@@ -1070,14 +1070,14 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>1.1801</v>
+        <v>1.1619</v>
       </c>
       <c r="D39" t="n">
-        <v>2565873</v>
+        <v>2526191</v>
       </c>
     </row>
     <row r="40">
@@ -1088,14 +1088,14 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>2.3476</v>
+        <v>2.3128</v>
       </c>
       <c r="D40" t="n">
-        <v>47200339</v>
+        <v>46481585</v>
       </c>
     </row>
     <row r="41">
@@ -1106,14 +1106,14 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>2.3266</v>
+        <v>2.292</v>
       </c>
       <c r="D41" t="n">
-        <v>155242467</v>
+        <v>153000174</v>
       </c>
     </row>
     <row r="42">
@@ -1124,14 +1124,14 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>2.3307</v>
+        <v>2.2962</v>
       </c>
       <c r="D42" t="n">
-        <v>377114950</v>
+        <v>371573320</v>
       </c>
     </row>
     <row r="43">
@@ -1142,14 +1142,14 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>2.3626</v>
+        <v>2.3289</v>
       </c>
       <c r="D43" t="n">
-        <v>480857177</v>
+        <v>473974390</v>
       </c>
     </row>
     <row r="44">
@@ -1160,14 +1160,14 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>2.0391</v>
+        <v>2.0196</v>
       </c>
       <c r="D44" t="n">
-        <v>393620386</v>
+        <v>389760718</v>
       </c>
     </row>
     <row r="45">
@@ -1178,14 +1178,14 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>1.5548</v>
+        <v>1.5462</v>
       </c>
       <c r="D45" t="n">
-        <v>294503324</v>
+        <v>292027629</v>
       </c>
     </row>
     <row r="46">
@@ -1196,14 +1196,14 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>1.2134</v>
+        <v>1.2087</v>
       </c>
       <c r="D46" t="n">
-        <v>58226459</v>
+        <v>58083644</v>
       </c>
     </row>
     <row r="47">
@@ -1221,14 +1221,14 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>1.1389</v>
+        <v>1.1194</v>
       </c>
       <c r="D48" t="n">
-        <v>3755721.97</v>
+        <v>3684949.21</v>
       </c>
     </row>
     <row r="49">
@@ -1239,14 +1239,14 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>2.1417</v>
+        <v>2.1083</v>
       </c>
       <c r="D49" t="n">
-        <v>83948772.52</v>
+        <v>82675842.75</v>
       </c>
     </row>
     <row r="50">
@@ -1257,14 +1257,14 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>2.1606</v>
+        <v>2.1266</v>
       </c>
       <c r="D50" t="n">
-        <v>269986593.2</v>
+        <v>265722392.32</v>
       </c>
     </row>
     <row r="51">
@@ -1275,14 +1275,14 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>2.1784</v>
+        <v>2.1441</v>
       </c>
       <c r="D51" t="n">
-        <v>411711586.5</v>
+        <v>405199363.07</v>
       </c>
     </row>
     <row r="52">
@@ -1293,14 +1293,14 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>2.1816</v>
+        <v>2.1494</v>
       </c>
       <c r="D52" t="n">
-        <v>501328438.3</v>
+        <v>493905901.26</v>
       </c>
     </row>
     <row r="53">
@@ -1311,14 +1311,14 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>1.9678</v>
+        <v>1.9491</v>
       </c>
       <c r="D53" t="n">
-        <v>468010624.1</v>
+        <v>463508263.09</v>
       </c>
     </row>
     <row r="54">
@@ -1329,14 +1329,14 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>1.5442</v>
+        <v>1.5353</v>
       </c>
       <c r="D54" t="n">
-        <v>368167097.8</v>
+        <v>366178131.11</v>
       </c>
     </row>
     <row r="55">
@@ -1347,14 +1347,14 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>1.2046</v>
+        <v>1.1983</v>
       </c>
       <c r="D55" t="n">
-        <v>68503948.73999999</v>
+        <v>67984412.33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>